<commit_message>
feat: CRUD groupes gestionnaire + import avec affectation automatique groupe
- Ajoute GroupeController (store, update, destroy) avec routes gestionnaire
- Route GET /groupes migree vers GroupeController#index (supprime la closure)
- Etend ImportCompteService : colonne groupe optionnelle, creation automatique
  du groupe si inexistant (recherche insensible a la casse + trim)
- Met a jour les fixtures CSV/XLSX avec la colonne groupe

Closes #59
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/test-import.xlsx
+++ b/backend/tests/fixtures/test-import.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -34,6 +34,9 @@
     <t xml:space="preserve">role</t>
   </si>
   <si>
+    <t xml:space="preserve">groupe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Dupont</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
   </si>
   <si>
     <t xml:space="preserve">etudiant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LP DAWII</t>
   </si>
   <si>
     <t xml:space="preserve">Martin</t>
@@ -70,6 +76,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -129,8 +136,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -257,55 +272,61 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10.33"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: race condition si plusieurs lignes avec le même nom de groupe
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/test-import.xlsx
+++ b/backend/tests/fixtures/test-import.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="20">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -62,6 +62,24 @@
   </si>
   <si>
     <t xml:space="preserve">enseignant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biscard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">paulo.biscard@test.cometudiant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quentin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dupuy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qunetin@test.com</t>
   </si>
 </sst>
 </file>
@@ -71,7 +89,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -93,6 +111,13 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -136,12 +161,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -272,7 +305,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.27"/>
@@ -329,7 +362,45 @@
         <v>13</v>
       </c>
     </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" display="paulo.biscard@test.cometudiant"/>
+    <hyperlink ref="C5" r:id="rId2" display="qunetin@test.com"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>